<commit_message>
Update catalogue naming, F@ctory Express pricing notes, and Jet-Off N PDF
- Rename A-800C catalogue entry to JET-GUN A-800C (EN/JA) and move it
  to the top of the Oilkey Products section
- Remove unit-of-ten discount wording from all F@ctory Express E-price
  notes, page intros, and download disclaimers
- Drop the 10,000 JPY grease gun price from the sizes note
- Update LS-600E related-product row: E-price 8,000 -> 5,800, item
  no. 2118 -> 2113
- Replace Jet-Off N product sheet with the latest PDF (120KB -> 515KB)
- Regenerate F@ctory Express PDF/Excel downloads

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/factory-express-catalogue-en.xlsx
+++ b/public/downloads/factory-express-catalogue-en.xlsx
@@ -522,14 +522,14 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Issued: 2026-07-18</t>
+          <t>Issued: 2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>The E-price is the unit price (JPY) for an order of one; discounted pricing applies to orders in units of ten. Prices and lead times are subject to change without notice.</t>
+          <t>The E-price is the unit price (JPY) for an order of one. Prices and lead times are subject to change without notice.</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>*5 E-price — the price for an order quantity of one (JPY). Discounted prices apply to orders in units of ten; please enquire using the fax quote request form.</t>
+          <t>*5 E-price — the price for an order quantity of one (JPY). Please enquire using the fax quote request form.</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>*4 E-price — the price for an order quantity of one (JPY). Discounted prices apply to orders in units of ten; please enquire using the fax quote request form.</t>
+          <t>*4 E-price — the price for an order quantity of one (JPY). Please enquire using the fax quote request form.</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>*2 E-price — the price for an order quantity of one (JPY). Discounted prices apply to orders in units of ten; please enquire using the fax quote request form.</t>
+          <t>*2 E-price — the price for an order quantity of one (JPY). Please enquire using the fax quote request form.</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5225,7 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>*3 E-price — the price for an order quantity of one (JPY). Discounted prices apply to orders in units of ten; please enquire using the fax quote request form.</t>
+          <t>*3 E-price — the price for an order quantity of one (JPY). Please enquire using the fax quote request form.</t>
         </is>
       </c>
     </row>
@@ -5962,14 +5962,14 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>*2 Sizes — 400 g items come as cylindrical cartridges (10 per box). A dedicated grease gun is required for use; sold separately at 10,000 JPY.</t>
+          <t>*2 Sizes — 400 g items come as cylindrical cartridges (10 per box). A dedicated grease gun is required for use.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>*3 E-price — the price for an order quantity of one (JPY). Discounted prices apply to orders in units of ten; please enquire using the fax quote request form.</t>
+          <t>*3 E-price — the price for an order quantity of one (JPY). Please enquire using the fax quote request form.</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>*2 E-price — the price for an order quantity of one (JPY). Discounted prices apply to orders in units of ten; please enquire using the fax quote request form.</t>
+          <t>*2 E-price — the price for an order quantity of one (JPY). Please enquire using the fax quote request form.</t>
         </is>
       </c>
     </row>
@@ -6745,7 +6745,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2118</t>
+          <t>2113</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>8,000</t>
+          <t>5,800</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
@@ -6820,7 +6820,7 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>*1 E-price — the price for an order quantity of one (JPY). Discounted prices apply to orders of ten or more; please enquire using the fax quote request form.</t>
+          <t>*1 E-price — the price for an order quantity of one (JPY). Please enquire using the fax quote request form.</t>
         </is>
       </c>
     </row>

</xml_diff>